<commit_message>
Updated logic of Adminpage
</commit_message>
<xml_diff>
--- a/notification_configs/01_daily_status_reminders.xlsx
+++ b/notification_configs/01_daily_status_reminders.xlsx
@@ -670,7 +670,7 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>2025-09-11 02:47:34</t>
+          <t>2025-09-11 10:17:41</t>
         </is>
       </c>
     </row>
@@ -768,7 +768,7 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>2025-09-11 02:47:34</t>
+          <t>2025-09-11 10:17:41</t>
         </is>
       </c>
     </row>
@@ -866,7 +866,7 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>2025-09-11 02:47:34</t>
+          <t>2025-09-11 10:17:41</t>
         </is>
       </c>
     </row>
@@ -964,7 +964,7 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>2025-09-11 02:47:34</t>
+          <t>2025-09-11 10:17:41</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>2025-09-11 02:47:34</t>
+          <t>2025-09-11 10:17:41</t>
         </is>
       </c>
     </row>
@@ -1160,7 +1160,7 @@
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>2025-09-11 02:47:34</t>
+          <t>2025-09-11 10:17:41</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Added notification config files propreluy
</commit_message>
<xml_diff>
--- a/notification_configs/01_daily_status_reminders.xlsx
+++ b/notification_configs/01_daily_status_reminders.xlsx
@@ -125,8 +125,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="DailyStatusReminders" displayName="DailyStatusReminders" ref="A1:U10" headerRowCount="1">
-  <autoFilter ref="A1:U10"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="DailyStatusReminders" displayName="DailyStatusReminders" ref="A1:U6" headerRowCount="1">
+  <autoFilter ref="A1:U6"/>
   <tableColumns count="21">
     <tableColumn id="1" name="Primary_Key"/>
     <tableColumn id="2" name="Contact_Email"/>
@@ -443,11 +443,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U10"/>
+  <dimension ref="A1:U6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="29" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
@@ -579,37 +579,37 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>VENDOR_01111_20250911</t>
+          <t>VENDOR_EMP001_20250911</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>thunderblunder018@gmail.com</t>
+          <t>john.vendor@company.com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Gopal</t>
+          <t>John Smith</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>01111</t>
+          <t>EMP001</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>DEV</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>MEdiatek</t>
+          <t>TechCorp Solutions</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>MTK34710</t>
+          <t>M001</t>
         </is>
       </c>
       <c r="H2" t="n">
@@ -640,12 +640,12 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Please submit your daily attendance status - Gopal</t>
+          <t>Please submit your daily attendance status - John Smith</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>vendor_01111</t>
+          <t>vendor_emp001</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -670,29 +670,29 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>2025-09-11 19:08:12</t>
+          <t>2025-09-11 22:16:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>VENDOR_EMP001_20250911</t>
+          <t>VENDOR_EMP002_20250911</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>john.vendor@company.com</t>
+          <t>jane.vendor@company.com</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>John Smith</t>
+          <t>Jane Wilson</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>EMP001</t>
+          <t>EMP002</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -738,12 +738,12 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Please submit your daily attendance status - John Smith</t>
+          <t>Please submit your daily attendance status - Jane Wilson</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>vendor_emp001</t>
+          <t>vendor_emp002</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -768,44 +768,44 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>2025-09-11 19:08:12</t>
+          <t>2025-09-11 22:16:31</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>VENDOR_EMP002_20250911</t>
+          <t>VENDOR_EMP003_20250911</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>jane.vendor@company.com</t>
+          <t>mike.vendor@company.com</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Jane Wilson</t>
+          <t>Mike Rodriguez</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>EMP002</t>
+          <t>EMP003</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Operations</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>TechCorp Solutions</t>
+          <t>InfraCorp Ltd</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>M001</t>
+          <t>M002</t>
         </is>
       </c>
       <c r="H4" t="n">
@@ -836,12 +836,12 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Please submit your daily attendance status - Jane Wilson</t>
+          <t>Please submit your daily attendance status - Mike Rodriguez</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>vendor_emp002</t>
+          <t>vendor_emp003</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -866,44 +866,44 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>2025-09-11 19:08:12</t>
+          <t>2025-09-11 22:16:31</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>VENDOR_EMP003_20250911</t>
+          <t>VENDOR_EMP004_20250911</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>mike.vendor@company.com</t>
+          <t>sarah.vendor@company.com</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Mike Rodriguez</t>
+          <t>Sarah Parker</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>EMP003</t>
+          <t>EMP004</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>Quality Assurance</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>InfraCorp Ltd</t>
+          <t>QualityCorp Inc</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>M002</t>
+          <t>M003</t>
         </is>
       </c>
       <c r="H5" t="n">
@@ -934,12 +934,12 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Please submit your daily attendance status - Mike Rodriguez</t>
+          <t>Please submit your daily attendance status - Sarah Parker</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>vendor_emp003</t>
+          <t>vendor_emp004</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
@@ -964,44 +964,44 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>2025-09-11 19:08:12</t>
+          <t>2025-09-11 22:16:31</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>VENDOR_EMP004_20250911</t>
+          <t>VENDOR_EMP005_20250911</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>sarah.vendor@company.com</t>
+          <t>david.vendor@company.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Sarah Parker</t>
+          <t>David Kim</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>EMP004</t>
+          <t>EMP005</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Quality Assurance</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>QualityCorp Inc</t>
+          <t>TechCorp Solutions</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>M003</t>
+          <t>M001</t>
         </is>
       </c>
       <c r="H6" t="n">
@@ -1032,12 +1032,12 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Please submit your daily attendance status - Sarah Parker</t>
+          <t>Please submit your daily attendance status - David Kim</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>vendor_emp004</t>
+          <t>vendor_emp005</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -1062,387 +1062,7 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>2025-09-11 19:08:12</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>VENDOR_EMP005_20250911</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>david.vendor@company.com</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>David Kim</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>EMP005</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Engineering</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>TechCorp Solutions</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>M001</t>
-        </is>
-      </c>
-      <c r="H7" t="n">
-        <v>3</v>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="K7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>Please submit your daily attendance status - David Kim</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>vendor_emp005</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>EMAIL,TEAMS</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="T7" t="inlineStr">
-        <is>
-          <t>2025-09-11</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>2025-09-11 19:08:12</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>VENDOR_OT1_20250911</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>ot1@vendor.com</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>abc1</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>OT1</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>WCS/MSE7</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Vendor Company</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="n">
-        <v>3</v>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="K8" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>Please submit your daily attendance status - abc1</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>vendor_ot1</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>EMAIL,TEAMS</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="T8" t="inlineStr">
-        <is>
-          <t>2025-09-11</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>2025-09-11 19:08:12</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>VENDOR_OT2_20250911</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>ot2@vendor.com</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>abc2</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>OT2</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>WCS/MSE7</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Vendor Company</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="n">
-        <v>3</v>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="K9" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>Please submit your daily attendance status - abc2</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>vendor_ot2</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>EMAIL,TEAMS</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="S9" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="T9" t="inlineStr">
-        <is>
-          <t>2025-09-11</t>
-        </is>
-      </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>2025-09-11 19:08:12</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>VENDOR_OT3_20250911</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>ot3@vendor.com</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>abc3</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>OT3</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>WCS/MSE8</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Vendor Company</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="n">
-        <v>3</v>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="K10" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>Please submit your daily attendance status - abc3</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>vendor_ot3</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>EMAIL,TEAMS</t>
-        </is>
-      </c>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="T10" t="inlineStr">
-        <is>
-          <t>2025-09-11</t>
-        </is>
-      </c>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>2025-09-11 19:08:12</t>
+          <t>2025-09-11 22:16:31</t>
         </is>
       </c>
     </row>

</xml_diff>